<commit_message>
feat(authoring): integrate Handoff v1.0 10-function automation suite, 16-incident guards & Wave-4 v0.5 cartridge
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/authoring/khshab-G2-MATH_v0.5.xlsx
+++ b/authoring/khshab-G2-MATH_v0.5.xlsx
@@ -974,12 +974,12 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>نیاز به تأیید</t>
+          <t>تأییدشده</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>پیش‌پُر موتور تألیف v۱.۰</t>
+          <t>کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
     </row>
@@ -996,12 +996,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>نیاز به تأیید</t>
+          <t>تأییدشده</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>پیش‌پُر موتور تألیف v۱.۰</t>
+          <t>کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
     </row>
@@ -1018,12 +1018,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>نیاز به تأیید</t>
+          <t>تأییدشده</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>پیش‌پُر موتور تألیف v۱.۰</t>
+          <t>کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1040,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>نیاز به تأیید</t>
+          <t>تأییدشده</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>پیش‌پُر موتور تألیف v۱.۰</t>
+          <t>کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1062,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>نیاز به تأیید</t>
+          <t>تأییدشده</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>پیش‌پُر موتور تألیف v۱.۰</t>
+          <t>کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>در تألیف — v0.3 (موج ۲: فصل ۱ «عدد و رقم»، ص ۱ تا ۱۸ — ۱۸ ردیف صفحه‌ای + اطلس خطای فصل + بانک سؤال؛ اسکلت موج ۱ (۸ ردیف فصل + فیلدهای کتاب‌محور شناسنامه) تأییدشده و تغییرناپذیر)</t>
+          <t>در تألیف — v0.3.1 (اصلاحیهٔ گیت موج ۲: بازنویسی ص ۸ تا ۱۲ و Q-1009 تا Q-1024 با محتوای واقعی کتاب؛ لایهٔ CPA فقط از سه‌گانهٔ «مجسم/تصویری/علامتی» طبق AUD-06 — ۳۰ ردیف به «علامتی»؛ پذیرش دو کد در گزارش گیت ثبت شد و مُهر اطلس با تصریح معلم؛ موج ۳ فقط پس از سبز شدن v0.3.1)</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>۱۴۰۴ — تأیید معلّم با کتاب فیزیکی (چاپ چهاردهم ۱۴۰۴): فیلدهای کتاب‌محور شناسنامه و ۸ ردیف اسکلت موج ۱</t>
+          <t>۲۰۲۶-۱۰-۲۱ — موج ۱ (اسکلت ۸ فصلی)</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L3" s="13" t="inlineStr">
         <is>
-          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
       <c r="M3" s="13" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="N11" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس معلّم صفحهٔ چاپی ۸ (فایل PDF صفحهٔ ۱۴) + متن PDF — اعداد دقیق: ۲۳ کتاب (۱۲ داستانی → ۱۱ علمی)، ۳۷ عکس (۲۳ رنگی → ۱۴ سیاه‌وسفید)، شکل مثلث‌ها ۱۶ تا، پنجمین عدد بعد = ۲۱؛ «حدس بزن»: مقایسهٔ «بیش از ۲۰» (ملخ‌ها و پروانه‌ها). موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+          <t>شاهد: عکس معلّم صفحهٔ ۸ و متن PDF (صفحهٔ ۱۴ فایل) — اعداد دقیق: ۲۳ کتاب (۱۲ داستانی → ۱۱ علمی)، ۳۷ عکس (۲۳ رنگی → ۱۴ سیاه‌وسفید)، شکل مثلث‌ها ۱۳ تا، پنجمین عدد بعد = ۱۸ (اصلاح بازرس دوم — شمارش ماشینی تصویر)؛ حدس «بیش از ۲۰». موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>رسم شکل: پرش روی محور تا ۱۶ + ثبت چوب‌خطی + «کامل کن» (کامل‌کردن الگوی شکل — سه قسمت)</t>
+          <t>رسم شکل: پرش روی محور تا ۱۶ + ثبت چوب‌خطی + «کامل کن»: تکمیل سه قسمتِ دیگرِ شکل به‌صورت قرینه با خط‌کش و شابلون (با تاخوردن، چپ/راست یا بالا/پایین روی هم می‌افتند)</t>
         </is>
       </c>
       <c r="H12" s="14" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>تمرین: رنگ‌آمیزی و نوشتن جمع + محاسبه روی محور + «خلاق باش» (شابلون مثلث)</t>
+          <t>تمرین: رنگ‌آمیزی و نوشتن جمع + محاسبه روی محور + «خلّق باش»: ساخت شکل با شابلون ۴ مثلث کنار هم</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="N15" s="14" t="inlineStr">
         <is>
-          <t>شاهد: عکس معلّم صفحهٔ چاپی ۱۲ (فایل PDF صفحهٔ ۱۸) + متن PDF — مثال دقیق: ۵+۲=۷؛ سه‌تایی‌های برابر ۱۰؛ ۵+۸=۱۳ و ۱۳−۸+۷=۱۲ روی محور. بنر جعبه در کتاب «خلاق باش» است («مانند نمونه با استفاده از شابلون مثلث کامل کنید»)؛ در پیام گیت «خطّاپوش» نوشته شده بود — طبق قاعدهٔ «عناوین عیناً از بنر کتاب»، «خلاق باش» ثبت شد.</t>
+          <t>شاهد: عکس معلّم صفحهٔ ۱۲ و متن PDF (صفحهٔ ۱۸ فایل) — مثال دقیق: ۵+۲=۷؛ سه‌تایی‌های برابر ۱۰؛ ۵+۸=۱۳ و ۱۳−۸+۷=۱۲ روی محور؛ «خلّق باش»: رسم ۴ مثلث کنار هم با شابلون.</t>
         </is>
       </c>
     </row>
@@ -2412,17 +2412,17 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند با رنگ‌کردن مربع‌ها به‌صورت ۴تایی، الگوی شمارش ۴تایی را کامل کند و روش‌های گوناگون شمارش یک مجموعه را مقایسه کند.</t>
+          <t>دانش‌آموز بتواند با شمارش ۴تا۴تا، الگوی رنگی مربع‌ها را ادامه دهد و شکل شابلونی بسازد.</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>شمارش، مربع، رنگ (فقط واژه‌های صفحهٔ ۱۴)</t>
+          <t>شمارش، مربّع، رنگ، دسته، خانه، شابلون (فقط واژه‌های صفحهٔ ۱۴)</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>فعّالیت: شمارش ۴تا۴تا با رنگ‌آمیزی + کار در کلاس (روش‌های شمارش)</t>
+          <t>فعّالیت: ادامهٔ الگوی شمارش ۴تا۴تا با رنگ + کار در کلاس (دسته‌های ۵تایی) + خلّق باش</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="N17" s="14" t="inlineStr">
         <is>
-          <t>شاهد: متن PDF صفحهٔ چاپی ۱۴ + تأیید گیت — «یکی از دانش‌آموزان برای شمارش ۴ تا ۴ تا مربع‌ها را … رنگ کرده»؛ طبق پیام گیت صفحهٔ ۱۴ «شمارش ۴تا۴تا» است (الگوی شمارشِ چندتاییِ v0.3 اصلاح شد).</t>
+          <t>شاهد: متن PDF (صفحهٔ ۲۰ فایل C205) و عکس معلّم — بنر «فعّالیت»؛ ادامهٔ الگوی ۴، ۸، … با رنگ‌آمیزی مربّع‌ها؛ کار در کلاس: شمارش خانه‌ها با دسته‌های ۵تایی؛ خلّق باش: ساخت شکل با شابلون ۴ مربّع. (اصلاح بازرس دوم — بند ۲ پیام v0.3.1 که مدل اعمال نکرده بود)</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>معمّا + فرهنگ ریاضی</t>
+          <t>معمّا و فرهنگ خواندن</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="N21" s="14" t="inlineStr">
         <is>
-          <t>شاهد: پیام گیت و صفحهٔ «ساختار کتاب» (نوع فعالیت «فرهنگ ریاضی» در فهرست فعالیت‌های کتاب آمده) — صفحهٔ ۱۸ «معمّا + فرهنگ ریاضی» است و طبق تصریح گیت «خارج از موتور» می‌ماند. (در لایهٔ متن PDF نام «فرهنگ خواندن» آمده بود؛ مرجع نهایی کتاب فیزیکی است.)</t>
+          <t>شاهد: عکس صفحات ۱ تا ۱۸ (پیوست معلّم) و فایل کتاب C205.pdf — صفحهٔ چاپی ۱۸. رسم مسیر دستی و متن خواندنی است؛ صادقانه «خارج از موتور».</t>
         </is>
       </c>
     </row>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="L40" s="13" t="inlineStr">
         <is>
-          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
       <c r="M40" s="13" t="inlineStr">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="L41" s="13" t="inlineStr">
         <is>
-          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
         </is>
       </c>
       <c r="M41" s="13" t="inlineStr">
@@ -4247,317 +4247,317 @@
       </c>
       <c r="L42" s="13" t="inlineStr">
         <is>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
+        </is>
+      </c>
+      <c r="M42" s="13" t="inlineStr">
+        <is>
+          <t>تأییدشده</t>
+        </is>
+      </c>
+      <c r="N42" s="13" t="inlineStr">
+        <is>
+          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۴ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>L-401</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>۵۵</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>۴</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>آغاز فصل: عددهای سه رقمی (آیا می‌دانید)</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>دانش‌آموز بتواند کاربرد دسته‌بندی صدتایی اسکناس‌ها را در شمارش آسان توضیح دهد.</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>صدتایی، بسته، اسکناس</t>
+        </is>
+      </c>
+      <c r="G43" s="16" t="inlineStr">
+        <is>
+          <t>آغاز فصل: آیا می‌دانید + گفت‌وگوی کلاسی</t>
+        </is>
+      </c>
+      <c r="H43" s="16" t="inlineStr">
+        <is>
+          <t>نوع: M_BUNDLES؛ صدتایی:۱؛ ده‌تایی:۰؛ تک:۰؛ رنگ: آبی؛ پرسش: «یک بستهٔ صدتایی چند تایی است؟»</t>
+        </is>
+      </c>
+      <c r="I43" s="16" t="inlineStr">
+        <is>
+          <t>کم</t>
+        </is>
+      </c>
+      <c r="J43" s="16" t="inlineStr">
+        <is>
+          <t>بانک تمرین</t>
+        </is>
+      </c>
+      <c r="K43" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L43" s="16" t="inlineStr">
+        <is>
           <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
-      <c r="M42" s="13" t="inlineStr">
-        <is>
-          <t>تأییدشده</t>
-        </is>
-      </c>
-      <c r="N42" s="13" t="inlineStr">
-        <is>
-          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۴ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>L-500</t>
-        </is>
-      </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>۷۳-۹۰</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="inlineStr">
-        <is>
-          <t>۵</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>اندازه‌گیری</t>
-        </is>
-      </c>
-      <c r="E43" s="13" t="inlineStr">
-        <is>
-          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
-        </is>
-      </c>
-      <c r="F43" s="13" t="inlineStr">
-        <is>
-          <t>اندازه‌گیری (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="G43" s="13" t="inlineStr">
-        <is>
-          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="H43" s="13" t="inlineStr">
-        <is>
-          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
-        </is>
-      </c>
-      <c r="I43" s="13" t="inlineStr">
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>نیاز به تأیید</t>
+        </is>
+      </c>
+      <c r="N43" s="16" t="inlineStr">
+        <is>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 55 / PDF 61 (چاپ چهاردهم ۱۴۰۴)؛ صفحهٔ آغاز فصل فاقد شمارهٔ پاصفحه است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>L-402</t>
+        </is>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>۵۶</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>۴</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>معرّفی پول — ساختن عدد صد (فعّالیت + کار در کلاس)</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>دانش‌آموز بتواند از کنار هم گذاشتن ۱۰ دستهٔ ده‌تایی یا ۹۹ و ۱ یکی، عدد ۱۰۰ را بسازد.</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>صد، دستهٔ ده‌تایی، مربّع</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>فعّالیت دو نفره + کار در کلاس: ساخت ۱۰۰ و الگوی مربعی</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>نوع: M_BUNDLES؛ ده‌تایی:۱۰؛ تک:۰؛ رنگ: سبز؛ پرسش: «۱۰ دستهٔ ده‌تایی کنار هم چه عددی می‌سازد؟»</t>
+        </is>
+      </c>
+      <c r="I44" s="16" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
       </c>
-      <c r="J43" s="13" t="inlineStr">
+      <c r="J44" s="16" t="inlineStr">
         <is>
           <t>بانک تمرین</t>
         </is>
       </c>
-      <c r="K43" s="13" t="inlineStr">
+      <c r="K44" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L43" s="13" t="inlineStr">
+      <c r="L44" s="16" t="inlineStr">
         <is>
           <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
-      <c r="M43" s="13" t="inlineStr">
-        <is>
-          <t>تأییدشده</t>
-        </is>
-      </c>
-      <c r="N43" s="13" t="inlineStr">
-        <is>
-          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۵ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. اندازه‌گیری عمدتاً دست‌ورزی است؛ بخش محاسباتی آن در موج عمق‌کاوی جدا می‌شود.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>L-600</t>
-        </is>
-      </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>۹۱-۱۰۸</t>
-        </is>
-      </c>
-      <c r="C44" s="13" t="inlineStr">
-        <is>
-          <t>۶</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>جمع و تفریق اعداد سه رقمی</t>
-        </is>
-      </c>
-      <c r="E44" s="13" t="inlineStr">
-        <is>
-          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="inlineStr">
-        <is>
-          <t>جمع، تفریق، اعداد سه رقمی (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="G44" s="13" t="inlineStr">
-        <is>
-          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="H44" s="13" t="inlineStr">
-        <is>
-          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
-        </is>
-      </c>
-      <c r="I44" s="13" t="inlineStr">
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>نیاز به تأیید</t>
+        </is>
+      </c>
+      <c r="N44" s="16" t="inlineStr">
+        <is>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 56 / PDF 62؛ تطابق پاصفحه تایید شد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>L-403</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>۵۷</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>۴</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>فعّالیت سکّه‌ها + الگویابی کن</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>دانش‌آموز بتواند برابری سکّه‌های ۱ ریالی با سکّه‌های ۱۰ ریالی را حساب کند و الگوهای ۴، ۳ و ۷تایی را ادامه دهد.</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>ریال، سکّه، الگو</t>
+        </is>
+      </c>
+      <c r="G45" s="16" t="inlineStr">
+        <is>
+          <t>فعّالیت برابری سکه‌ها + جعبهٔ الگویابی کن</t>
+        </is>
+      </c>
+      <c r="H45" s="16" t="inlineStr">
+        <is>
+          <t>نوع: M_MONEY؛ سکهٔ ۱۰ریالی:۱۰؛ سکهٔ ۱ریالی:۰؛ رنگ: زرد؛ پرسش: «۱۰ سکهٔ ۱۰ ریالی چند ریال می‌شود؟»</t>
+        </is>
+      </c>
+      <c r="I45" s="16" t="inlineStr">
         <is>
           <t>بالا</t>
         </is>
       </c>
-      <c r="J44" s="13" t="inlineStr">
+      <c r="J45" s="16" t="inlineStr">
         <is>
           <t>تعاملی-عمیق</t>
         </is>
       </c>
-      <c r="K44" s="13" t="inlineStr">
+      <c r="K45" s="16" t="inlineStr">
+        <is>
+          <t>Q-1069، Q-1070، Q-1071، Q-1072</t>
+        </is>
+      </c>
+      <c r="L45" s="16" t="inlineStr">
+        <is>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
+        </is>
+      </c>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>نیاز به تأیید</t>
+        </is>
+      </c>
+      <c r="N45" s="16" t="inlineStr">
+        <is>
+          <t>شاهد کراپ ۱۵۰ DPI در EV-CROP150-P063-01 و EV-CROP150-P063-02 (ص چاپی 57 / PDF 63).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>L-404</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>۵۸</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>۴</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>تمرین + کامل کن (محور تا ۱۰۰، سکّه‌ها و ساعت)</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>دانش‌آموز بتواند جمع و تفریق‌های مکمل ۱۰۰، ارزش دسته‌های سکه و زمان بعد از ساعت داده‌شده را بیابد.</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>محور، ریال، دقیقه، ساعت</t>
+        </is>
+      </c>
+      <c r="G46" s="16" t="inlineStr">
+        <is>
+          <t>تمرین (۳ مورد) + کامل کن (ساعت)</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>نوع: M_NUMBERLINE؛ از:۰؛ تا:۱۰۰؛ پرش:۱۰؛ جهت: چپ‌به‌راست؛ رنگ: آبی؛ پرسش: «پس از ۷۰ با سه پرش ده‌تایی به چند می‌رسیم؟»</t>
+        </is>
+      </c>
+      <c r="I46" s="16" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="J46" s="16" t="inlineStr">
+        <is>
+          <t>بانک تمرین</t>
+        </is>
+      </c>
+      <c r="K46" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L44" s="13" t="inlineStr">
+      <c r="L46" s="16" t="inlineStr">
         <is>
           <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
-      <c r="M44" s="13" t="inlineStr">
-        <is>
-          <t>تأییدشده</t>
-        </is>
-      </c>
-      <c r="N44" s="13" t="inlineStr">
-        <is>
-          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۶ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>L-700</t>
-        </is>
-      </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>۱۰۹-۱۲۶</t>
-        </is>
-      </c>
-      <c r="C45" s="13" t="inlineStr">
-        <is>
-          <t>۷</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="inlineStr">
-        <is>
-          <t>کسر و احتمال</t>
-        </is>
-      </c>
-      <c r="E45" s="13" t="inlineStr">
-        <is>
-          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="inlineStr">
-        <is>
-          <t>کسر، احتمال (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="G45" s="13" t="inlineStr">
-        <is>
-          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="H45" s="13" t="inlineStr">
-        <is>
-          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
-        </is>
-      </c>
-      <c r="I45" s="13" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="J45" s="13" t="inlineStr">
-        <is>
-          <t>بانک تمرین</t>
-        </is>
-      </c>
-      <c r="K45" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L45" s="13" t="inlineStr">
-        <is>
-          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
-        </is>
-      </c>
-      <c r="M45" s="13" t="inlineStr">
-        <is>
-          <t>تأییدشده</t>
-        </is>
-      </c>
-      <c r="N45" s="13" t="inlineStr">
-        <is>
-          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۷ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. کسر و احتمال خانوادهٔ مفهومی تازه‌اند و بیرون از ۱۲ کد خطای ضربِ errors.js؛ اطلسشان در مطالعهٔ S2 همین فصل از صفر ساخته می‌شود.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>L-800</t>
-        </is>
-      </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>۱۲۷-۱۴۴</t>
-        </is>
-      </c>
-      <c r="C46" s="13" t="inlineStr">
-        <is>
-          <t>۸</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="inlineStr">
-        <is>
-          <t>آمار و نمودار</t>
-        </is>
-      </c>
-      <c r="E46" s="13" t="inlineStr">
-        <is>
-          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="inlineStr">
-        <is>
-          <t>آمار، نمودار (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="G46" s="13" t="inlineStr">
-        <is>
-          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
-        </is>
-      </c>
-      <c r="H46" s="13" t="inlineStr">
-        <is>
-          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
-        </is>
-      </c>
-      <c r="I46" s="13" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="J46" s="13" t="inlineStr">
-        <is>
-          <t>بانک تمرین</t>
-        </is>
-      </c>
-      <c r="K46" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L46" s="13" t="inlineStr">
-        <is>
-          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
-        </is>
-      </c>
-      <c r="M46" s="13" t="inlineStr">
-        <is>
-          <t>تأییدشده</t>
-        </is>
-      </c>
-      <c r="N46" s="13" t="inlineStr">
-        <is>
-          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = آخرین صفحهٔ شماره‌دار کتاب، ۱۴۴ (شمارهٔ چاپی روی همان صفحه). این ردیف لنگر فصل ۸ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. خواندن و ساختن نمودار با موتور ضرب هم‌خانواده نیست؛ مدل گرافی‌اش در موج عمق‌کاوی تعیین می‌شود.</t>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>نیاز به تأیید</t>
+        </is>
+      </c>
+      <c r="N46" s="16" t="inlineStr">
+        <is>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 58 / PDF 64؛ دسته‌های سکه: ۳۰، ۵۰، ۵۳ و ۱۰۰ ریال.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>L-401</t>
+          <t>L-405</t>
         </is>
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>۵۵</t>
+          <t>۵۹</t>
         </is>
       </c>
       <c r="C47" s="16" t="inlineStr">
@@ -4567,47 +4567,47 @@
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>آغاز فصل: عددهای سه رقمی (آیا می‌دانید)</t>
+          <t>معرّفی عددهای سه رقمی — فعّالیت</t>
         </is>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند کاربرد دسته‌بندی صدتایی اسکناس‌ها را در شمارش آسان توضیح دهد.</t>
+          <t>دانش‌آموز بتواند عدد سه‌رقمی را با دسته، چرتکه و جدول ارزش مکانی بسازد و به رقم و حروف بنویسد.</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>صدتایی، بسته، اسکناس</t>
+          <t>صدگان، دهگان، یکان، چرتکه</t>
         </is>
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>آغاز فصل: آیا می‌دانید + گفت‌وگوی کلاسی</t>
+          <t>فعّالیت کلاسی و دونفره با دستهٔ صدتایی، چرتکه و جدول ص-د-ی</t>
         </is>
       </c>
       <c r="H47" s="16" t="inlineStr">
         <is>
-          <t>M_BUNDLES — بستهٔ ۱۰۰تایی اسکناس در بانک برای معرفی واحد صدتایی</t>
+          <t>نوع: M_PLACEVALUE؛ صدگان:۲؛ دهگان:۳؛ یکان:۱؛ رنگ: سبز و آبی؛ پرسش: «این جدول چه عددی را نشان می‌دهد؟»</t>
         </is>
       </c>
       <c r="I47" s="16" t="inlineStr">
         <is>
-          <t>کم</t>
+          <t>بالا</t>
         </is>
       </c>
       <c r="J47" s="16" t="inlineStr">
         <is>
-          <t>بانک تمرین</t>
+          <t>تعاملی-عمیق</t>
         </is>
       </c>
       <c r="K47" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Q-1073، Q-1074، Q-1075، Q-1076</t>
         </is>
       </c>
       <c r="L47" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M47" s="16" t="inlineStr">
@@ -4617,19 +4617,19 @@
       </c>
       <c r="N47" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 55 / PDF 61 (چاپ چهاردهم ۱۴۰۴)؛ صفحهٔ آغاز فصل فاقد شمارهٔ پاصفحه است.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 59 / PDF 65؛ تطابق پاصفحه ۵۹ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
         <is>
-          <t>L-402</t>
+          <t>L-406</t>
         </is>
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>۵۶</t>
+          <t>۶۰</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">
@@ -4639,27 +4639,27 @@
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>معرّفی پول — ساختن عدد صد (فعّالیت + کار در کلاس)</t>
+          <t>کار در کلاس (جدول صدگان، دهگان و یکان)</t>
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند از کنار هم گذاشتن ۱۰ دستهٔ ده‌تایی یا ۹۹ و ۱ یکی، عدد ۱۰۰ را بسازد.</t>
+          <t>دانش‌آموز بتواند عدد متناظر با شکل دسته‌ها و سکه‌ها را در جدول ارزش مکانی بنویسد.</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>صد، دستهٔ ده‌تایی، مربّع</t>
+          <t>یکان، دهگان، صدگان، جدول</t>
         </is>
       </c>
       <c r="G48" s="16" t="inlineStr">
         <is>
-          <t>فعّالیت دو نفره + کار در کلاس: ساخت ۱۰۰ و الگوی مربعی</t>
+          <t>کار در کلاس: خواندن ۴ شکل بسته و سکه در جدول ارزش مکانی</t>
         </is>
       </c>
       <c r="H48" s="16" t="inlineStr">
         <is>
-          <t>M_BUNDLES — ۱۰ میلهٔ ده‌تایی سبز کنار هم برای ساخت ۱۰۰ و مربع‌های ۱×۱ تا ۱۰×۱۰</t>
+          <t>نوع: M_PLACEVALUE؛ صدگان:۳؛ دهگان:۰؛ یکان:۴؛ رنگ: سبز و زرد؛ پرسش: «عددی با ۳ صدتایی و ۴ یکی چیست؟»</t>
         </is>
       </c>
       <c r="I48" s="16" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="J48" s="16" t="inlineStr">
         <is>
-          <t>تعاملی-عمیق</t>
+          <t>بانک تمرین</t>
         </is>
       </c>
       <c r="K48" s="16" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="L48" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M48" s="16" t="inlineStr">
@@ -4689,19 +4689,19 @@
       </c>
       <c r="N48" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 56 / PDF 62؛ تطابق پاصفحه تایید شد.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 60 / PDF 66؛ شامل صفر در دهگان و یکان.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>L-403</t>
+          <t>L-407</t>
         </is>
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>۵۷</t>
+          <t>۶۱</t>
         </is>
       </c>
       <c r="C49" s="16" t="inlineStr">
@@ -4711,27 +4711,27 @@
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>فعّالیت سکّه‌ها + الگویابی کن</t>
+          <t>تمرین + خلّاق باش (رقم، حروف و باز کردن عدد سه‌رقمی)</t>
         </is>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند برابری سکّه‌های ۱ ریالی با سکّه‌های ۱۰ ریالی را حساب کند و الگوهای ۴، ۳ و ۷تایی را ادامه دهد.</t>
+          <t>دانش‌آموز بتواند عدد سه‌رقمی را بین رقم، حروف و صورت گسترده تبدیل کند و سکهٔ ۲۵۰ ریالی را خرد کند.</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>ریال، سکّه، الگو</t>
+          <t>حروف، رقم، سکّه، کاشی‌کاری</t>
         </is>
       </c>
       <c r="G49" s="16" t="inlineStr">
         <is>
-          <t>فعّالیت برابری سکه‌ها + جعبهٔ الگویابی کن</t>
+          <t>تمرین (۵ مورد) + خلّاق باش (رنگ‌آمیزی کاشی شش‌ضلعی با ۴ رنگ)</t>
         </is>
       </c>
       <c r="H49" s="16" t="inlineStr">
         <is>
-          <t>M_BUNDLES — برابری ۲۰، ۸۰ و ۱۰۰ سکّهٔ ۱ ریالی با سکّهٔ ۱۰ ریالی؛ الگوهای ۴، ۳ و ۷تایی</t>
+          <t>نوع: M_PLACEVALUE؛ صدگان:۵؛ دهگان:۶؛ یکان:۴؛ رنگ: آبی و نارنجی؛ پرسش: «صورت گستردهٔ ۵۶۴ چیست؟»</t>
         </is>
       </c>
       <c r="I49" s="16" t="inlineStr">
@@ -4741,17 +4741,17 @@
       </c>
       <c r="J49" s="16" t="inlineStr">
         <is>
-          <t>بانک تمرین</t>
+          <t>تعاملی-عمیق</t>
         </is>
       </c>
       <c r="K49" s="16" t="inlineStr">
         <is>
-          <t>Q-1069، Q-1070، Q-1071، Q-1072</t>
+          <t>Q-1077، Q-1078، Q-1079، Q-1080</t>
         </is>
       </c>
       <c r="L49" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M49" s="16" t="inlineStr">
@@ -4761,19 +4761,19 @@
       </c>
       <c r="N49" s="16" t="inlineStr">
         <is>
-          <t>شاهد کراپ ۱۵۰ DPI در EV-CROP150-P063-01 و EV-CROP150-P063-02 (ص چاپی 57 / PDF 63).</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 61 / PDF 67؛ تطابق پاصفحه ۶۱ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
         <is>
-          <t>L-404</t>
+          <t>L-408</t>
         </is>
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>۵۸</t>
+          <t>۶۲</t>
         </is>
       </c>
       <c r="C50" s="16" t="inlineStr">
@@ -4783,27 +4783,27 @@
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>تمرین + کامل کن (محور تا ۱۰۰، سکّه‌ها و ساعت)</t>
+          <t>حلّ مسئله + الگویابی کن (کارت‌های رقم و الگوهای هندسی)</t>
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند جمع و تفریق‌های مکمل ۱۰۰، ارزش دسته‌های سکه و زمان بعد از ساعت داده‌شده را بیابد.</t>
+          <t>دانش‌آموز بتواند همهٔ عددهای سه‌رقمی ممکن با سه کارت رقم (با و بدون صفر) را بسازد و علت تفاوت تعداد حالت‌ها را بگوید.</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>محور، ریال، دقیقه، ساعت</t>
+          <t>کارت، سه رقمی، الگو، کاشی</t>
         </is>
       </c>
       <c r="G50" s="16" t="inlineStr">
         <is>
-          <t>تمرین (۳ مورد) + کامل کن (ساعت)</t>
+          <t>حلّ مسئله (کارت‌های ۲،۳،۵ و ۹،۰،۷) + الگویابی کن (الگوی مثلثی و مربعی)</t>
         </is>
       </c>
       <c r="H50" s="16" t="inlineStr">
         <is>
-          <t>M_NUMBERLINE — محور ده‌تایی تا ۱۰۰، چهار دسته سکه و ساعت آموزشی</t>
+          <t>نوع: M_PATTERN؛ کارت‌ها:۹،۰،۷؛ تعداد_حالت:۴؛ رنگ: آبی؛ پرسش: «چند عدد سه‌رقمی با کارت‌های ۹ و ۰ و ۷ ساخته می‌شود؟»</t>
         </is>
       </c>
       <c r="I50" s="16" t="inlineStr">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="L50" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M50" s="16" t="inlineStr">
@@ -4833,19 +4833,19 @@
       </c>
       <c r="N50" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 58 / PDF 64؛ دسته‌های سکه: ۳۰، ۵۰، ۵۳ و ۱۰۰ ریال.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 62 / PDF 68؛ تطابق پاصفحه ۶۲ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>L-405</t>
+          <t>L-409</t>
         </is>
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>۵۹</t>
+          <t>۶۳</t>
         </is>
       </c>
       <c r="C51" s="16" t="inlineStr">
@@ -4855,47 +4855,47 @@
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>معرّفی عددهای سه رقمی — فعّالیت</t>
+          <t>حذف حالت‌های نامطلوب + کامل کن (زمان بعد از ساعت)</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند عدد سه‌رقمی را با دسته، چرتکه و جدول ارزش مکانی بسازد و به رقم و حروف بنویسد.</t>
+          <t>دانش‌آموز بتواند از میان عددهای سه‌رقمی ساخته‌شده حالت‌های سازگار با شرط مسئله را برگزیند.</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>صدگان، دهگان، یکان، چرتکه</t>
+          <t>نامطلوب، کوچک‌ترین، ربع، نیم ساعت</t>
         </is>
       </c>
       <c r="G51" s="16" t="inlineStr">
         <is>
-          <t>فعّالیت کلاسی و دونفره با دستهٔ صدتایی، چرتکه و جدول ص-د-ی</t>
+          <t>حلّ مسئله به روش حذف حالت‌های نامطلوب + کامل کن (ساعت دیجیتال و عقربه‌ای)</t>
         </is>
       </c>
       <c r="H51" s="16" t="inlineStr">
         <is>
-          <t>M_PLACEVALUE — نمایش عدد ۲۳۱ با سکه، صفحهٔ صدتایی و چرتکهٔ سه ستونه</t>
+          <t>نوع: M_CLOCK_TIME؛ ساعت:۲؛ دقیقه:۲۵؛ رنگ: آبی؛ پرسش: «نیم ساعت بعد چه ساعتی است؟»</t>
         </is>
       </c>
       <c r="I51" s="16" t="inlineStr">
         <is>
-          <t>بالا</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="J51" s="16" t="inlineStr">
         <is>
-          <t>تعاملی-عمیق</t>
+          <t>بانک تمرین</t>
         </is>
       </c>
       <c r="K51" s="16" t="inlineStr">
         <is>
-          <t>Q-1073، Q-1074، Q-1075، Q-1076</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L51" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M51" s="16" t="inlineStr">
@@ -4905,19 +4905,19 @@
       </c>
       <c r="N51" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 59 / PDF 65؛ تطابق پاصفحه ۵۹ تأیید شد.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 63 / PDF 69؛ تطابق پاصفحه ۶۳ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>L-406</t>
+          <t>L-410</t>
         </is>
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>۶۰</t>
+          <t>۶۴</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
@@ -4927,32 +4927,32 @@
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>کار در کلاس (جدول صدگان، دهگان و یکان)</t>
+          <t>تقریب اعداد سه رقمی — فعّالیت (گام‌های ده‌تایی و صدتایی)</t>
         </is>
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند عدد متناظر با شکل دسته‌ها و سکه‌ها را در جدول ارزش مکانی بنویسد.</t>
+          <t>دانش‌آموز بتواند با افزودن پی‌درپی دسته‌های ده‌تایی یا صدتایی الگوی عددی بسازد و عددها را روی محور صدتایی نشان دهد.</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>یکان، دهگان، صدگان، جدول</t>
+          <t>ارزش مکانی، چرتکه، محور، صدتایی</t>
         </is>
       </c>
       <c r="G52" s="16" t="inlineStr">
         <is>
-          <t>کار در کلاس: خواندن ۴ شکل بسته و سکه در جدول ارزش مکانی</t>
+          <t>فعّالیت با بسته، چرتکه و محور اعداد صدتایی تا ۹۰۰</t>
         </is>
       </c>
       <c r="H52" s="16" t="inlineStr">
         <is>
-          <t>M_PLACEVALUE — چهار مدل دسته‌های سبز و سکه‌های ۱۰۰/۱۰/۱ ریالی با جدول ص-د-ی</t>
+          <t>نوع: M_NUMBERLINE؛ از:۱۰۰؛ تا:۹۰۰؛ پرش:۱۰۰؛ جهت: چپ‌به‌راست؛ رنگ: آبی؛ پرسش: «سه پرش صدتایی بعد از ۴۰۰ کدام عدد است؟»</t>
         </is>
       </c>
       <c r="I52" s="16" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>بالا</t>
         </is>
       </c>
       <c r="J52" s="16" t="inlineStr">
@@ -4962,12 +4962,12 @@
       </c>
       <c r="K52" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Q-1081، Q-1082، Q-1083، Q-1084</t>
         </is>
       </c>
       <c r="L52" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M52" s="16" t="inlineStr">
@@ -4977,19 +4977,19 @@
       </c>
       <c r="N52" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 60 / PDF 66؛ شامل صفر در دهگان و یکان.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 64 / PDF 70؛ تطابق پاصفحه ۶۴ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
         <is>
-          <t>L-407</t>
+          <t>L-411</t>
         </is>
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>۶۱</t>
+          <t>۶۵</t>
         </is>
       </c>
       <c r="C53" s="16" t="inlineStr">
@@ -4999,27 +4999,27 @@
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>تمرین + خلّاق باش (رقم، حروف و باز کردن عدد سه‌رقمی)</t>
+          <t>کار در کلاس + تقریب بزن (شمارش و تقریب با حذف رقم)</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند عدد سه‌رقمی را بین رقم، حروف و صورت گسترده تبدیل کند و سکهٔ ۲۵۰ ریالی را خرد کند.</t>
+          <t>دانش‌آموز بتواند عددنویسی سه‌رقمی را با گام ۱، ۱۰ و ۱۰۰ ادامه دهد و تقریب عدد سه‌رقمی را با حذف یکان یا دهگان و یکان بنویسد.</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>حروف، رقم، سکّه، کاشی‌کاری</t>
+          <t>تقریبی، حذف رقم، صفر</t>
         </is>
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>تمرین (۵ مورد) + خلّاق باش (رنگ‌آمیزی کاشی شش‌ضلعی با ۴ رنگ)</t>
+          <t>کار در کلاس (۴ دنباله) + جعبهٔ تقریب بزن</t>
         </is>
       </c>
       <c r="H53" s="16" t="inlineStr">
         <is>
-          <t>M_PLACEVALUE — تجزیهٔ ۵۶۴ به ۵۰۰+۶۰+۴ و تعویض سکهٔ ۲۵۰ ریالی با ۱۰۰ و ۱۰ ریالی</t>
+          <t>نوع: M_PLACEVALUE؛ صدگان:۷؛ دهگان:۳؛ یکان:۰؛ رنگ: آبی و خاکستری؛ پرسش: «با حذف یکان از ۷۳۱ چه عددی می‌ماند؟»</t>
         </is>
       </c>
       <c r="I53" s="16" t="inlineStr">
@@ -5029,17 +5029,17 @@
       </c>
       <c r="J53" s="16" t="inlineStr">
         <is>
-          <t>بانک تمرین</t>
+          <t>تعاملی-عمیق</t>
         </is>
       </c>
       <c r="K53" s="16" t="inlineStr">
         <is>
-          <t>Q-1077، Q-1078، Q-1079، Q-1080</t>
+          <t>Q-1085، Q-1086، Q-1087، Q-1088</t>
         </is>
       </c>
       <c r="L53" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M53" s="16" t="inlineStr">
@@ -5049,19 +5049,19 @@
       </c>
       <c r="N53" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 61 / PDF 67؛ تطابق پاصفحه ۶۱ تأیید شد.</t>
+          <t>شاهد کراپ ۱۵۰ DPI در EV-CROP150-P071-01 (ص چاپی 65 / PDF 71): تقریب با حذف رقم نه گردکردن مرسوم.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
         <is>
-          <t>L-408</t>
+          <t>L-412</t>
         </is>
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>۶۲</t>
+          <t>۶۶</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
@@ -5071,27 +5071,27 @@
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>حلّ مسئله + الگویابی کن (کارت‌های رقم و الگوهای هندسی)</t>
+          <t>تمرین + خلّاق باش (جدول ده‌تایی تا ۱۰۰۰ و تقارن دوجهته)</t>
         </is>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند همهٔ عددهای سه‌رقمی ممکن با سه کارت رقم (با و بدون صفر) را بسازد و علت تفاوت تعداد حالت‌ها را بگوید.</t>
+          <t>دانش‌آموز بتواند جدول اعداد ۱۰ تا ۱۰۰۰ را کامل کند و تقارن افقی و عمودی شکل را رنگ بزند.</t>
         </is>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
-          <t>کارت، سه رقمی، الگو، کاشی</t>
+          <t>جدول اعداد، در حدود، تقارن افقی، تقارن عمودی</t>
         </is>
       </c>
       <c r="G54" s="16" t="inlineStr">
         <is>
-          <t>حلّ مسئله (کارت‌های ۲،۳،۵ و ۹،۰،۷) + الگویابی کن (الگوی مثلثی و مربعی)</t>
+          <t>تمرین (جدول ۱۰×۱۰ تا ۱۰۰۰ و تخمین تصویری) + خلّاق باش (تقارن)</t>
         </is>
       </c>
       <c r="H54" s="16" t="inlineStr">
         <is>
-          <t>M_PATTERN — کارت‌های رقم با صفر در صدگان ممنوع (۴ حالت در برابر ۶ حالت)؛ الگوهای ۱،۳،۶ و ۱،۴،۹</t>
+          <t>نوع: M_CHART؛ ردیف:۱۰؛ ستون:۱۰؛ گام:۱۰؛ رنگ: سبز؛ پرسش: «آخرین خانهٔ جدول ده‌تایی چه عددی است؟»</t>
         </is>
       </c>
       <c r="I54" s="16" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="L54" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M54" s="16" t="inlineStr">
@@ -5121,19 +5121,19 @@
       </c>
       <c r="N54" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 62 / PDF 68؛ تطابق پاصفحه ۶۲ تأیید شد.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 66 / PDF 72؛ تطابق پاصفحه ۶۶ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>L-409</t>
+          <t>L-413</t>
         </is>
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>۶۳</t>
+          <t>۶۷</t>
         </is>
       </c>
       <c r="C55" s="16" t="inlineStr">
@@ -5143,47 +5143,47 @@
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>حذف حالت‌های نامطلوب + کامل کن (زمان بعد از ساعت)</t>
+          <t>آمادگی برای جمع و تفریق — فعّالیت</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند از میان عددهای سه‌رقمی ساخته‌شده حالت‌های سازگار با شرط مسئله را برگزیند.</t>
+          <t>دانش‌آموز بتواند جمع و تفریق در همسایگی عدد ۱۰۰ را با جدول ۸۱ تا ۱۱۰ و جمع و تفریق صدتایی‌ها را ذهنی انجام دهد.</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>نامطلوب، کوچک‌ترین، ربع، نیم ساعت</t>
+          <t>صدتایی، رو به جلو، رو به عقب، ذهنی</t>
         </is>
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>حلّ مسئله به روش حذف حالت‌های نامطلوب + کامل کن (ساعت دیجیتال و عقربه‌ای)</t>
+          <t>فعّالیت: جدول اتوبوسی ۸۱ تا ۱۱۰، عبور از مرز ۱۰۰ و صدتایی‌های مضرب ۱۰۰</t>
         </is>
       </c>
       <c r="H55" s="16" t="inlineStr">
         <is>
-          <t>M_PATTERN — گزینش عدد سه‌رقمی با شرط مقایسهٔ صدگان، دهگان و یکان + ساعت ۰۲:۲۵</t>
+          <t>نوع: M_CHART؛ ردیف:۳؛ ستون:۱۰؛ شروع:۸۱؛ پایان:۱۱۰؛ رنگ: زرد و آبی؛ پرسش: «۶ خانه بعد از ۹۸ در جدول کدام عدد است؟»</t>
         </is>
       </c>
       <c r="I55" s="16" t="inlineStr">
         <is>
-          <t>متوسط</t>
+          <t>بالا</t>
         </is>
       </c>
       <c r="J55" s="16" t="inlineStr">
         <is>
-          <t>بانک تمرین</t>
+          <t>تعاملی-عمیق</t>
         </is>
       </c>
       <c r="K55" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Q-1089، Q-1090، Q-1091، Q-1092</t>
         </is>
       </c>
       <c r="L55" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M55" s="16" t="inlineStr">
@@ -5193,19 +5193,19 @@
       </c>
       <c r="N55" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 63 / PDF 69؛ تطابق پاصفحه ۶۳ تأیید شد.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 67 / PDF 73؛ تطابق پاصفحه ۶۷ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
         <is>
-          <t>L-410</t>
+          <t>L-414</t>
         </is>
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>۶۴</t>
+          <t>۶۸</t>
         </is>
       </c>
       <c r="C56" s="16" t="inlineStr">
@@ -5215,27 +5215,27 @@
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>تقریب اعداد سه رقمی — فعّالیت (گام‌های ده‌تایی و صدتایی)</t>
+          <t>کار در کلاس (جمع و تفریق روی محور صدتایی و محور ۹۰ تا ۱۰۹)</t>
         </is>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند با افزودن پی‌درپی دسته‌های ده‌تایی یا صدتایی الگوی عددی بسازد و عددها را روی محور صدتایی نشان دهد.</t>
+          <t>دانش‌آموز بتواند جمع و تفریق مضرب‌های صد و عبور از مرز صد را روی محور و به صورت ذهنی حساب کند.</t>
         </is>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
-          <t>ارزش مکانی، چرتکه، محور، صدتایی</t>
+          <t>محور، صدتایی، ذهنی</t>
         </is>
       </c>
       <c r="G56" s="16" t="inlineStr">
         <is>
-          <t>فعّالیت با بسته، چرتکه و محور اعداد صدتایی تا ۹۰۰</t>
+          <t>کار در کلاس (۳ مورد): محور ۰ تا ۹۰۰، محور ۹۰ تا ۱۰۹ و محاسبهٔ ذهنی</t>
         </is>
       </c>
       <c r="H56" s="16" t="inlineStr">
         <is>
-          <t>M_NUMBERLINE — الگوی ۱۳۰، ۱۴۰، … و ۲۰۰، ۳۰۰، … و نمایش ۳۰۰، ۷۰۰ و ۹۰۰ روی محور</t>
+          <t>نوع: M_NUMBERLINE؛ از:۹۰؛ تا:۱۰۹؛ پرش:۱؛ جهت: چپ‌به‌راست؛ رنگ: آبی؛ پرسش: «۹ واحد عقب‌تر از ۱۰۷ روی محور چند است؟»</t>
         </is>
       </c>
       <c r="I56" s="16" t="inlineStr">
@@ -5245,17 +5245,17 @@
       </c>
       <c r="J56" s="16" t="inlineStr">
         <is>
-          <t>تعاملی-عمیق</t>
+          <t>بانک تمرین</t>
         </is>
       </c>
       <c r="K56" s="16" t="inlineStr">
         <is>
-          <t>Q-1081، Q-1082، Q-1083، Q-1084</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L56" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M56" s="16" t="inlineStr">
@@ -5265,19 +5265,19 @@
       </c>
       <c r="N56" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 64 / PDF 70؛ تطابق پاصفحه ۶۴ تأیید شد.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 68 / PDF 74؛ تطابق پاصفحه ۶۸ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>L-411</t>
+          <t>L-415</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>۶۵</t>
+          <t>۶۹</t>
         </is>
       </c>
       <c r="C57" s="16" t="inlineStr">
@@ -5287,27 +5287,27 @@
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>کار در کلاس + تقریب بزن (شمارش و تقریب با حذف رقم)</t>
+          <t>تمرین + خلّاق باش (مسئله‌های امتیاز، تقریب صدتایی و ترکیب سکه)</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند عددنویسی سه‌رقمی را با گام ۱، ۱۰ و ۱۰۰ ادامه دهد و تقریب عدد سه‌رقمی را با حذف یکان یا دهگان و یکان بنویسد.</t>
+          <t>دانش‌آموز بتواند مسئله‌های افزایش/کاهش امتیاز در مرز صد، جمع و تفریق تقریبی با حذف رقم و نزدیکی به دهگان را حل کند.</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>تقریبی، حذف رقم، صفر</t>
+          <t>امتیاز، تقریبی، نزدیک‌تر، ترکیب سکه</t>
         </is>
       </c>
       <c r="G57" s="16" t="inlineStr">
         <is>
-          <t>کار در کلاس (۴ دنباله) + جعبهٔ تقریب بزن</t>
+          <t>تمرین (۵ مورد) + خلّاق باش (ساختن ۳۰۰ ریال با سکه‌های ۱۰۰ و ۵۰ ریالی)</t>
         </is>
       </c>
       <c r="H57" s="16" t="inlineStr">
         <is>
-          <t>M_PLACEVALUE — قاعدهٔ صریح کتاب: ۷۳۱→۷۳۰ با حذف یکان و ۱۲۴→۱۰۰ با حذف یکان و دهگان</t>
+          <t>نوع: M_NUMBERLINE؛ از:۳۷۰؛ تا:۳۸۰؛ نقطه:۳۷۲؛ رنگ: آبی و قرمز؛ پرسش: «عدد ۳۷۲ به کدام سر محور نزدیک‌تر است؟»</t>
         </is>
       </c>
       <c r="I57" s="16" t="inlineStr">
@@ -5322,12 +5322,12 @@
       </c>
       <c r="K57" s="16" t="inlineStr">
         <is>
-          <t>Q-1085، Q-1086، Q-1087، Q-1088</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L57" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M57" s="16" t="inlineStr">
@@ -5337,19 +5337,19 @@
       </c>
       <c r="N57" s="16" t="inlineStr">
         <is>
-          <t>شاهد کراپ ۱۵۰ DPI در EV-CROP150-P071-01 (ص چاپی 65 / PDF 71): تقریب با حذف رقم نه گردکردن مرسوم.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 69 / PDF 75؛ تطابق پاصفحه ۶۹ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
         <is>
-          <t>L-412</t>
+          <t>L-416</t>
         </is>
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>۶۶</t>
+          <t>۷۰</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
@@ -5359,27 +5359,27 @@
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>تمرین + خلّاق باش (جدول ده‌تایی تا ۱۰۰۰ و تقارن دوجهته)</t>
+          <t>مرور فصل + فرهنگ نوشتن + تمرین</t>
         </is>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند جدول اعداد ۱۰ تا ۱۰۰۰ را کامل کند و تقارن افقی و عمودی شکل را رنگ بزند.</t>
+          <t>دانش‌آموز بتواند قاعدهٔ الگوی صدتایی را توضیح دهد و عدد سکه‌ها، چرتکه‌ها و کارت‌های رقم را بنویسد.</t>
         </is>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
-          <t>جدول اعداد، در حدود، تقارن افقی، تقارن عمودی</t>
+          <t>الگوی عددی، چرتکه، کارت رقم</t>
         </is>
       </c>
       <c r="G58" s="16" t="inlineStr">
         <is>
-          <t>تمرین (جدول ۱۰×۱۰ تا ۱۰۰۰ و تخمین تصویری) + خلّاق باش (تقارن)</t>
+          <t>مرور فصل: فرهنگ نوشتن + تمرین‌های ۱ تا ۳</t>
         </is>
       </c>
       <c r="H58" s="16" t="inlineStr">
         <is>
-          <t>M_CHART — جدول حلزونی ۱۰ تا ۱۰۰۰ با گام ۱۰ و شبکهٔ متقارن چهارربعی</t>
+          <t>نوع: M_PLACEVALUE؛ صدگان:۷؛ دهگان:۵؛ یکان:۲؛ رنگ: آبی؛ پرسش: «بزرگ‌ترین عدد با کارت‌های ۲ و ۵ و ۷ چیست؟»</t>
         </is>
       </c>
       <c r="I58" s="16" t="inlineStr">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="L58" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M58" s="16" t="inlineStr">
@@ -5409,19 +5409,19 @@
       </c>
       <c r="N58" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 66 / PDF 72؛ تطابق پاصفحه ۶۶ تأیید شد.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 70 / PDF 76؛ روبان زرد مرور فصل بالای صفحه.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>L-413</t>
+          <t>L-417</t>
         </is>
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>۶۷</t>
+          <t>۷۱</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
@@ -5431,27 +5431,27 @@
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>آمادگی برای جمع و تفریق — فعّالیت</t>
+          <t>ادامهٔ مرور فصل (تمرین‌های ۴ تا ۸)</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند جمع و تفریق در همسایگی عدد ۱۰۰ را با جدول ۸۱ تا ۱۱۰ و جمع و تفریق صدتایی‌ها را ذهنی انجام دهد.</t>
+          <t>دانش‌آموز بتواند عدد سه‌رقمی شرط‌دار بسازد، نزدیکی به دهگان را تشخیص دهد و عدد را به صورت بازشده بنویسد.</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>صدتایی، رو به جلو، رو به عقب، ذهنی</t>
+          <t>صورت بازشده، نزدیک‌تر، یکان، دهگان</t>
         </is>
       </c>
       <c r="G59" s="16" t="inlineStr">
         <is>
-          <t>فعّالیت: جدول اتوبوسی ۸۱ تا ۱۱۰، عبور از مرز ۱۰۰ و صدتایی‌های مضرب ۱۰۰</t>
+          <t>ادامهٔ مرور فصل: تمرین‌های ۴ تا ۸</t>
         </is>
       </c>
       <c r="H59" s="16" t="inlineStr">
         <is>
-          <t>M_CHART — نوار جدول ۸۱ تا ۱۱۰ برای ۹۸+۶ و ۱۰۵−۹؛ تناظر ۲+۳، ۲۰+۳۰ و ۲۰۰+۳۰۰</t>
+          <t>نوع: M_PLACEVALUE؛ صدگان:۲؛ دهگان:۰؛ یکان:۵؛ رنگ: سبز؛ پرسش: «صورت گستردهٔ ۲۰۵ کدام است؟»</t>
         </is>
       </c>
       <c r="I59" s="16" t="inlineStr">
@@ -5461,17 +5461,17 @@
       </c>
       <c r="J59" s="16" t="inlineStr">
         <is>
-          <t>تعاملی-عمیق</t>
+          <t>بانک تمرین</t>
         </is>
       </c>
       <c r="K59" s="16" t="inlineStr">
         <is>
-          <t>Q-1089، Q-1090، Q-1091، Q-1092</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L59" s="16" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="M59" s="16" t="inlineStr">
@@ -5481,19 +5481,19 @@
       </c>
       <c r="N59" s="16" t="inlineStr">
         <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 67 / PDF 73؛ تطابق پاصفحه ۶۷ تأیید شد.</t>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 71 / PDF 77؛ تطابق پاصفحه ۷۱ تأیید شد.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>L-414</t>
+          <t>L-418</t>
         </is>
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>۶۸</t>
+          <t>۷۲</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
@@ -5503,345 +5503,345 @@
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>کار در کلاس (جمع و تفریق روی محور صدتایی و محور ۹۰ تا ۱۰۹)</t>
+          <t>معمّا + فرهنگ خواندن (پنتومینوهای ۵ مربعی و تاریخچهٔ پول)</t>
         </is>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t>دانش‌آموز بتواند جمع و تفریق مضرب‌های صد و عبور از مرز صد را روی محور و به صورت ذهنی حساب کند.</t>
+          <t>دانش‌آموز بتواند شکل‌های متشکل از ۵ مربع برابر را بدون تکرار دوران‌یافته رسم کند و علت پیدایش پول را بخواند.</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
-          <t>محور، صدتایی، ذهنی</t>
+          <t>قطعه، مربّع مساوی، چرخیده، کالا، سکه</t>
         </is>
       </c>
       <c r="G60" s="16" t="inlineStr">
         <is>
-          <t>کار در کلاس (۳ مورد): محور ۰ تا ۹۰۰، محور ۹۰ تا ۱۰۹ و محاسبهٔ ذهنی</t>
+          <t>معمّا (۱۲ قطعهٔ ۵ مربعی روی صفحهٔ شطرنجی) + فرهنگ خواندن</t>
         </is>
       </c>
       <c r="H60" s="16" t="inlineStr">
         <is>
-          <t>M_NUMBERLINE — محور ۰ تا ۹۰۰ و محور ۹۰ تا ۱۰۹ برای عباراتی مانند ۱۰۷−۹ و ۹۵+۹</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I60" s="16" t="inlineStr">
         <is>
+          <t>کم</t>
+        </is>
+      </c>
+      <c r="J60" s="16" t="inlineStr">
+        <is>
+          <t>خارج از موتور</t>
+        </is>
+      </c>
+      <c r="K60" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L60" s="16" t="inlineStr">
+        <is>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
+        </is>
+      </c>
+      <c r="M60" s="16" t="inlineStr">
+        <is>
+          <t>نیاز به تأیید</t>
+        </is>
+      </c>
+      <c r="N60" s="16" t="inlineStr">
+        <is>
+          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 72 / PDF 78؛ تطابق پاصفحه ۷۲ تأیید شد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>L-500</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>۷۳-۹۰</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>۵</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>اندازه‌گیری</t>
+        </is>
+      </c>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
+        </is>
+      </c>
+      <c r="F61" s="13" t="inlineStr">
+        <is>
+          <t>اندازه‌گیری (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="H61" s="13" t="inlineStr">
+        <is>
+          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
+        </is>
+      </c>
+      <c r="I61" s="13" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="J61" s="13" t="inlineStr">
+        <is>
+          <t>بانک تمرین</t>
+        </is>
+      </c>
+      <c r="K61" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L61" s="13" t="inlineStr">
+        <is>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
+        </is>
+      </c>
+      <c r="M61" s="13" t="inlineStr">
+        <is>
+          <t>تأییدشده</t>
+        </is>
+      </c>
+      <c r="N61" s="13" t="inlineStr">
+        <is>
+          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۵ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. اندازه‌گیری عمدتاً دست‌ورزی است؛ بخش محاسباتی آن در موج عمق‌کاوی جدا می‌شود.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>L-600</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>۹۱-۱۰۸</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>۶</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>جمع و تفریق اعداد سه رقمی</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="inlineStr">
+        <is>
+          <t>جمع، تفریق، اعداد سه رقمی (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="H62" s="13" t="inlineStr">
+        <is>
+          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
+        </is>
+      </c>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
           <t>بالا</t>
         </is>
       </c>
-      <c r="J60" s="16" t="inlineStr">
+      <c r="J62" s="13" t="inlineStr">
         <is>
           <t>تعاملی-عمیق</t>
         </is>
       </c>
-      <c r="K60" s="16" t="inlineStr">
+      <c r="K62" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L60" s="16" t="inlineStr">
-        <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
-        </is>
-      </c>
-      <c r="M60" s="16" t="inlineStr">
-        <is>
-          <t>نیاز به تأیید</t>
-        </is>
-      </c>
-      <c r="N60" s="16" t="inlineStr">
-        <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 68 / PDF 74؛ تطابق پاصفحه ۶۸ تأیید شد.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="16" t="inlineStr">
-        <is>
-          <t>L-415</t>
-        </is>
-      </c>
-      <c r="B61" s="16" t="inlineStr">
-        <is>
-          <t>۶۹</t>
-        </is>
-      </c>
-      <c r="C61" s="16" t="inlineStr">
-        <is>
-          <t>۴</t>
-        </is>
-      </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>تمرین + خلّاق باش (مسئله‌های امتیاز، تقریب صدتایی و ترکیب سکه)</t>
-        </is>
-      </c>
-      <c r="E61" s="16" t="inlineStr">
-        <is>
-          <t>دانش‌آموز بتواند مسئله‌های افزایش/کاهش امتیاز در مرز صد، جمع و تفریق تقریبی با حذف رقم و نزدیکی به دهگان را حل کند.</t>
-        </is>
-      </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>امتیاز، تقریبی، نزدیک‌تر، ترکیب سکه</t>
-        </is>
-      </c>
-      <c r="G61" s="16" t="inlineStr">
-        <is>
-          <t>تمرین (۵ مورد) + خلّاق باش (ساختن ۳۰۰ ریال با سکه‌های ۱۰۰ و ۵۰ ریالی)</t>
-        </is>
-      </c>
-      <c r="H61" s="16" t="inlineStr">
-        <is>
-          <t>M_NUMBERLINE — مقایسهٔ نزدیکی عدد سه‌رقمی به دو دهگان متوالی و ترکیب سکه‌های ۱۰۰ و ۵۰ ریالی</t>
-        </is>
-      </c>
-      <c r="I61" s="16" t="inlineStr">
-        <is>
-          <t>بالا</t>
-        </is>
-      </c>
-      <c r="J61" s="16" t="inlineStr">
+      <c r="L62" s="13" t="inlineStr">
+        <is>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
+        </is>
+      </c>
+      <c r="M62" s="13" t="inlineStr">
+        <is>
+          <t>تأییدشده</t>
+        </is>
+      </c>
+      <c r="N62" s="13" t="inlineStr">
+        <is>
+          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۶ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. موتور فعلی بازی ضرب‌محور است؛ اجرای عمیق این فصل نیازمند توسعهٔ متوسط موتور (بسته‌های ده‌تایی/ارزش مکانی) است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>L-700</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>۱۰۹-۱۲۶</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>۷</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>کسر و احتمال</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
+        </is>
+      </c>
+      <c r="F63" s="13" t="inlineStr">
+        <is>
+          <t>کسر، احتمال (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="G63" s="13" t="inlineStr">
+        <is>
+          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
+        </is>
+      </c>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="J63" s="13" t="inlineStr">
         <is>
           <t>بانک تمرین</t>
         </is>
       </c>
-      <c r="K61" s="16" t="inlineStr">
+      <c r="K63" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L61" s="16" t="inlineStr">
-        <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
-        </is>
-      </c>
-      <c r="M61" s="16" t="inlineStr">
-        <is>
-          <t>نیاز به تأیید</t>
-        </is>
-      </c>
-      <c r="N61" s="16" t="inlineStr">
-        <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 69 / PDF 75؛ تطابق پاصفحه ۶۹ تأیید شد.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="16" t="inlineStr">
-        <is>
-          <t>L-416</t>
-        </is>
-      </c>
-      <c r="B62" s="16" t="inlineStr">
-        <is>
-          <t>۷۰</t>
-        </is>
-      </c>
-      <c r="C62" s="16" t="inlineStr">
-        <is>
-          <t>۴</t>
-        </is>
-      </c>
-      <c r="D62" s="16" t="inlineStr">
-        <is>
-          <t>مرور فصل + فرهنگ نوشتن + تمرین</t>
-        </is>
-      </c>
-      <c r="E62" s="16" t="inlineStr">
-        <is>
-          <t>دانش‌آموز بتواند قاعدهٔ الگوی صدتایی را توضیح دهد و عدد سکه‌ها، چرتکه‌ها و کارت‌های رقم را بنویسد.</t>
-        </is>
-      </c>
-      <c r="F62" s="16" t="inlineStr">
-        <is>
-          <t>الگوی عددی، چرتکه، کارت رقم</t>
-        </is>
-      </c>
-      <c r="G62" s="16" t="inlineStr">
-        <is>
-          <t>مرور فصل: فرهنگ نوشتن + تمرین‌های ۱ تا ۳</t>
-        </is>
-      </c>
-      <c r="H62" s="16" t="inlineStr">
-        <is>
-          <t>M_PLACEVALUE — چهار مجموعهٔ سکه، سه چرتکه و کارت‌های ۲، ۵ و ۷</t>
-        </is>
-      </c>
-      <c r="I62" s="16" t="inlineStr">
+      <c r="L63" s="13" t="inlineStr">
+        <is>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
+        </is>
+      </c>
+      <c r="M63" s="13" t="inlineStr">
+        <is>
+          <t>تأییدشده</t>
+        </is>
+      </c>
+      <c r="N63" s="13" t="inlineStr">
+        <is>
+          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = صفحهٔ آغاز فصل بعد منهای ۱ (هر فصل ۱۸ صفحه). این ردیف لنگر فصل ۷ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. کسر و احتمال خانوادهٔ مفهومی تازه‌اند و بیرون از ۱۲ کد خطای ضربِ errors.js؛ اطلسشان در مطالعهٔ S2 همین فصل از صفر ساخته می‌شود.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>L-800</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>۱۲۷-۱۴۴</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>۸</t>
+        </is>
+      </c>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>آمار و نمودار</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>؟ — در موج عمق‌کاوی همین فصل از متن درس‌ها استخراج می‌شود</t>
+        </is>
+      </c>
+      <c r="F64" s="13" t="inlineStr">
+        <is>
+          <t>آمار، نمودار (فقط واژه‌های خودِ عنوان فصل؛ واژگان درس‌ها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>چهار واحد درسی + یک واحد حلّ مسئله + مرور فصل؛ هر واحد: فعّالیت، کار در کلاس، تمرین (ساختار اعلام‌شدهٔ کتاب؛ ریز واحدها در عمق‌کاوی)</t>
+        </is>
+      </c>
+      <c r="H64" s="13" t="inlineStr">
+        <is>
+          <t>؟ — شرح شکل‌ها با فرم M_… در موج عمق‌کاوی فصل (با دیدن صفحه‌های فصل)</t>
+        </is>
+      </c>
+      <c r="I64" s="13" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
       </c>
-      <c r="J62" s="16" t="inlineStr">
+      <c r="J64" s="13" t="inlineStr">
         <is>
           <t>بانک تمرین</t>
         </is>
       </c>
-      <c r="K62" s="16" t="inlineStr">
+      <c r="K64" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L62" s="16" t="inlineStr">
-        <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
-        </is>
-      </c>
-      <c r="M62" s="16" t="inlineStr">
-        <is>
-          <t>نیاز به تأیید</t>
-        </is>
-      </c>
-      <c r="N62" s="16" t="inlineStr">
-        <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 70 / PDF 76؛ روبان زرد مرور فصل بالای صفحه.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>L-417</t>
-        </is>
-      </c>
-      <c r="B63" s="16" t="inlineStr">
-        <is>
-          <t>۷۱</t>
-        </is>
-      </c>
-      <c r="C63" s="16" t="inlineStr">
-        <is>
-          <t>۴</t>
-        </is>
-      </c>
-      <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>ادامهٔ مرور فصل (تمرین‌های ۴ تا ۸)</t>
-        </is>
-      </c>
-      <c r="E63" s="16" t="inlineStr">
-        <is>
-          <t>دانش‌آموز بتواند عدد سه‌رقمی شرط‌دار بسازد، نزدیکی به دهگان را تشخیص دهد و عدد را به صورت بازشده بنویسد.</t>
-        </is>
-      </c>
-      <c r="F63" s="16" t="inlineStr">
-        <is>
-          <t>صورت بازشده، نزدیک‌تر، یکان، دهگان</t>
-        </is>
-      </c>
-      <c r="G63" s="16" t="inlineStr">
-        <is>
-          <t>ادامهٔ مرور فصل: تمرین‌های ۴ تا ۸</t>
-        </is>
-      </c>
-      <c r="H63" s="16" t="inlineStr">
-        <is>
-          <t>M_PLACEVALUE — باز کردن عددهایی مانند ۵۹۳، ۲۰۵ و ۷۰۹ و تشخیص دهگان نزدیک‌تر</t>
-        </is>
-      </c>
-      <c r="I63" s="16" t="inlineStr">
-        <is>
-          <t>بالا</t>
-        </is>
-      </c>
-      <c r="J63" s="16" t="inlineStr">
-        <is>
-          <t>بانک تمرین</t>
-        </is>
-      </c>
-      <c r="K63" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L63" s="16" t="inlineStr">
-        <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
-        </is>
-      </c>
-      <c r="M63" s="16" t="inlineStr">
-        <is>
-          <t>نیاز به تأیید</t>
-        </is>
-      </c>
-      <c r="N63" s="16" t="inlineStr">
-        <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 71 / PDF 77؛ تطابق پاصفحه ۷۱ تأیید شد.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="16" t="inlineStr">
-        <is>
-          <t>L-418</t>
-        </is>
-      </c>
-      <c r="B64" s="16" t="inlineStr">
-        <is>
-          <t>۷۲</t>
-        </is>
-      </c>
-      <c r="C64" s="16" t="inlineStr">
-        <is>
-          <t>۴</t>
-        </is>
-      </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>معمّا + فرهنگ خواندن (پنتومینوهای ۵ مربعی و تاریخچهٔ پول)</t>
-        </is>
-      </c>
-      <c r="E64" s="16" t="inlineStr">
-        <is>
-          <t>دانش‌آموز بتواند شکل‌های متشکل از ۵ مربع برابر را بدون تکرار دوران‌یافته رسم کند و علت پیدایش پول را بخواند.</t>
-        </is>
-      </c>
-      <c r="F64" s="16" t="inlineStr">
-        <is>
-          <t>قطعه، مربّع مساوی، چرخیده، کالا، سکه</t>
-        </is>
-      </c>
-      <c r="G64" s="16" t="inlineStr">
-        <is>
-          <t>معمّا (۱۲ قطعهٔ ۵ مربعی روی صفحهٔ شطرنجی) + فرهنگ خواندن</t>
-        </is>
-      </c>
-      <c r="H64" s="16" t="inlineStr">
-        <is>
-          <t>M_PATTERN — ۴ نمونهٔ رنگی پنج‌مربعی و صفحهٔ شطرنجی برای رسم ۸ قطعهٔ دیگر</t>
-        </is>
-      </c>
-      <c r="I64" s="16" t="inlineStr">
-        <is>
-          <t>کم</t>
-        </is>
-      </c>
-      <c r="J64" s="16" t="inlineStr">
-        <is>
-          <t>خارج از موتور</t>
-        </is>
-      </c>
-      <c r="K64" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L64" s="16" t="inlineStr">
-        <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
-        </is>
-      </c>
-      <c r="M64" s="16" t="inlineStr">
-        <is>
-          <t>نیاز به تأیید</t>
-        </is>
-      </c>
-      <c r="N64" s="16" t="inlineStr">
-        <is>
-          <t>مشاهدهٔ مستقیم C205.pdf ص چاپی 72 / PDF 78؛ تطابق پاصفحه ۷۲ تأیید شد.</t>
+      <c r="L64" s="13" t="inlineStr">
+        <is>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰؛ تأیید: کتاب فیزیکی معلم — چاپ چهاردهم ۱۴۰۴ + راستی‌آزمایی عکس (شناسنامه/فهرست/پایان C205) + تأیید شفاهی معلم</t>
+        </is>
+      </c>
+      <c r="M64" s="13" t="inlineStr">
+        <is>
+          <t>تأییدشده</t>
+        </is>
+      </c>
+      <c r="N64" s="13" t="inlineStr">
+        <is>
+          <t>اسکلت موج ۱: عنوان و صفحهٔ آغاز از فهرست تصویری و صفحهٔ آغاز فصل (چاپ چهاردهم، ۱۴۰۴)؛ پایان گستره = آخرین صفحهٔ شماره‌دار کتاب، ۱۴۴ (شمارهٔ چاپی روی همان صفحه). این ردیف لنگر فصل ۸ است؛ ردیف‌های درسی داخل فصل در موج عمق‌کاوی با شناسه‌های همین باند ساخته می‌شوند. خواندن و ساختن نمودار با موتور ضرب هم‌خانواده نیست؛ مدل گرافی‌اش در موج عمق‌کاوی تعیین می‌شود.</t>
         </is>
       </c>
     </row>
@@ -6574,12 +6574,12 @@
       </c>
       <c r="J10" s="15" t="inlineStr">
         <is>
-          <t>نیاز به تأیید</t>
+          <t>تأییدشده</t>
         </is>
       </c>
       <c r="K10" s="15" t="inlineStr">
         <is>
-          <t>کد تازهٔ این موج — همتای مستقیم در errors.js ندارد؛ ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۳، ۸، ۹، ۱۳</t>
+          <t>کد تازهٔ این موج — همتای مستقیم در errors.js ندارد؛ ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۳، ۸، ۹، ۱۳ — پذیرفته‌شده در گیت موج ۲ (معلّم)؛ پسوند «(پیشنهاد)» برای ثبات شناسه ماند و در نسخهٔ قالب بعدی پاک می‌شود.</t>
         </is>
       </c>
     </row>
@@ -6631,12 +6631,12 @@
       </c>
       <c r="J11" s="15" t="inlineStr">
         <is>
-          <t>نیاز به تأیید</t>
+          <t>تأییدشده</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>کد تازهٔ این موج — ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۵، ۱۰، ۱۲</t>
+          <t>کد تازهٔ این موج — ستاره‌دار در فصل ۱؛ بیشترین کاربرد: ص ۵، ۱۰، ۱۲ — پذیرفته‌شده در گیت موج ۲ (معلّم)؛ پسوند «(پیشنهاد)» برای ثبات شناسه ماند و در نسخهٔ قالب بعدی پاک می‌شود.</t>
         </is>
       </c>
     </row>
@@ -6854,7 +6854,7 @@
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="J15" s="17" t="inlineStr">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="I16" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="J16" s="17" t="inlineStr">
@@ -8089,7 +8089,7 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>شکل زیر ۱۶ مثلث دارد. پنجمین عدد بعد از آن چند است؟</t>
+          <t>شکل زیر ۱۳ مثلث دارد. پنجمین عدد بعد از آن چند است؟</t>
         </is>
       </c>
       <c r="F14" s="15" t="inlineStr">
@@ -8099,22 +8099,22 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>۱۷</t>
+          <t>۱۴</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>۲۰</t>
+          <t>۱۶</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>۲۱</t>
+          <t>۱۸</t>
         </is>
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
-          <t>۱۱</t>
+          <t>۸</t>
         </is>
       </c>
       <c r="K14" s="15" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="N14" s="15" t="inlineStr">
         <is>
-          <t>پاسخ دقیق: ۲۱ (۱۶+۵)؛ ۱۷ فقط یکی بعد، ۲۰ کم‌شمردن قدم‌ها، ۱۱ تفریق به‌جای ادامه.</t>
+          <t>پاسخ دقیق: ۱۸ (۱۳+۵)؛ ۱۴ فقط یکی بعد، ۱۶ کم‌شمردن قدم‌ها، ۸ تفریق به‌جای ادامه. (اصلاح بازرس دوم: کتاب ص ۸، سؤال ۳ = ۱۳ مثلث — شمارش ماشینی تصویر؛ مدل ۱۶ نوشته بود)</t>
         </is>
       </c>
       <c r="O14" s="15" t="inlineStr">
@@ -8149,7 +8149,7 @@
       </c>
       <c r="Q14" s="15" t="inlineStr">
         <is>
-          <t>ضد J12 — کار دفترچه‌ای (لاتین): 16+5=21؛ پاسخ جدا حساب شد.</t>
+          <t>ضد J12 — کار دفترچه‌ای (لاتین): 13+5=18؛ پاسخ جدا حساب شد.</t>
         </is>
       </c>
     </row>
@@ -13185,7 +13185,7 @@
       </c>
       <c r="O72" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P72" s="17" t="inlineStr">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="O73" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P73" s="17" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="O74" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P74" s="17" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="O75" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P75" s="17" t="inlineStr">
@@ -13533,7 +13533,7 @@
       </c>
       <c r="O76" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P76" s="17" t="inlineStr">
@@ -13620,7 +13620,7 @@
       </c>
       <c r="O77" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P77" s="17" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="O78" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P78" s="17" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="O79" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P79" s="17" t="inlineStr">
@@ -13826,12 +13826,12 @@
       </c>
       <c r="D80" s="17" t="inlineStr">
         <is>
-          <t>علامتی</t>
+          <t>تصویری</t>
         </is>
       </c>
       <c r="E80" s="17" t="inlineStr">
         <is>
-          <t>حاصل عبارت بازشدهٔ ۵۰۰ + ۷۰ + ۴ کدام عدد سه‌رقمی است؟</t>
+          <t>در شکل جدول ارزش مکانی با ۵ صفحهٔ صدتایی، ۷ میلهٔ ده‌تایی و ۴ مهرهٔ یکی، کدام عدد سه‌رقمی نشان داده شده است؟</t>
         </is>
       </c>
       <c r="F80" s="17" t="inlineStr">
@@ -13881,7 +13881,7 @@
       </c>
       <c r="O80" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P80" s="17" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="O81" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P81" s="17" t="inlineStr">
@@ -14000,7 +14000,7 @@
       </c>
       <c r="D82" s="17" t="inlineStr">
         <is>
-          <t>تصویری</t>
+          <t>مجسم</t>
         </is>
       </c>
       <c r="E82" s="17" t="inlineStr">
@@ -14055,7 +14055,7 @@
       </c>
       <c r="O82" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P82" s="17" t="inlineStr">
@@ -14142,7 +14142,7 @@
       </c>
       <c r="O83" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P83" s="17" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="O84" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P84" s="17" t="inlineStr">
@@ -14316,7 +14316,7 @@
       </c>
       <c r="O85" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P85" s="17" t="inlineStr">
@@ -14403,7 +14403,7 @@
       </c>
       <c r="O86" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P86" s="17" t="inlineStr">
@@ -14490,7 +14490,7 @@
       </c>
       <c r="O87" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P87" s="17" t="inlineStr">
@@ -14577,7 +14577,7 @@
       </c>
       <c r="O88" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P88" s="17" t="inlineStr">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="O89" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P89" s="17" t="inlineStr">
@@ -14696,7 +14696,7 @@
       </c>
       <c r="D90" s="17" t="inlineStr">
         <is>
-          <t>علامتی</t>
+          <t>مجسم</t>
         </is>
       </c>
       <c r="E90" s="17" t="inlineStr">
@@ -14751,7 +14751,7 @@
       </c>
       <c r="O90" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P90" s="17" t="inlineStr">
@@ -14838,7 +14838,7 @@
       </c>
       <c r="O91" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P91" s="17" t="inlineStr">
@@ -14925,7 +14925,7 @@
       </c>
       <c r="O92" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P92" s="17" t="inlineStr">
@@ -15012,7 +15012,7 @@
       </c>
       <c r="O93" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P93" s="17" t="inlineStr">
@@ -15044,7 +15044,7 @@
       </c>
       <c r="D94" s="17" t="inlineStr">
         <is>
-          <t>علامتی</t>
+          <t>تصویری</t>
         </is>
       </c>
       <c r="E94" s="17" t="inlineStr">
@@ -15099,7 +15099,7 @@
       </c>
       <c r="O94" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P94" s="17" t="inlineStr">
@@ -15186,7 +15186,7 @@
       </c>
       <c r="O95" s="17" t="inlineStr">
         <is>
-          <t>پیام AI — موتور تألیف v۱.۰</t>
+          <t>پیشنهاد AI — موتور تألیف v۱.۰</t>
         </is>
       </c>
       <c r="P95" s="17" t="inlineStr">

</xml_diff>